<commit_message>
Update present perfect experience workbook
</commit_message>
<xml_diff>
--- a/Studymaterials/中学生英作文現在完了形_経験用法編.xlsx
+++ b/Studymaterials/中学生英作文現在完了形_経験用法編.xlsx
@@ -5833,7 +5833,7 @@
     <row r="18" ht="22" customHeight="1" s="6">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, you have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, you have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B18" s="27" t="n"/>
@@ -5849,7 +5849,7 @@
     <row r="19" ht="22" customHeight="1" s="6">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, you haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, you haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B19" s="27" t="n"/>
@@ -6009,7 +6009,7 @@
     <row r="29" ht="22" customHeight="1" s="6">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：You have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：You have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B29" s="27" t="n"/>
@@ -6025,7 +6025,7 @@
     <row r="30" ht="22" customHeight="1" s="6">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：You haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：You haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B30" s="27" t="n"/>
@@ -6295,7 +6295,7 @@
     <row r="47" ht="22" customHeight="1" s="6">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, I have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, I have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B47" s="27" t="n"/>
@@ -6311,7 +6311,7 @@
     <row r="48" ht="22" customHeight="1" s="6">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, I haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, I haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B48" s="27" t="n"/>
@@ -6471,7 +6471,7 @@
     <row r="58" ht="22" customHeight="1" s="6">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：I have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：I have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B58" s="27" t="n"/>
@@ -6487,7 +6487,7 @@
     <row r="59" ht="22" customHeight="1" s="6">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：I haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：I haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B59" s="27" t="n"/>
@@ -6757,7 +6757,7 @@
     <row r="76" ht="22" customHeight="1" s="6">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, he has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, he has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B76" s="27" t="n"/>
@@ -6773,7 +6773,7 @@
     <row r="77" ht="22" customHeight="1" s="6">
       <c r="A77" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, he hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, he hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B77" s="27" t="n"/>
@@ -6933,7 +6933,7 @@
     <row r="87" ht="22" customHeight="1" s="6">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：He has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：He has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B87" s="27" t="n"/>
@@ -6949,7 +6949,7 @@
     <row r="88" ht="22" customHeight="1" s="6">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：He hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：He hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B88" s="27" t="n"/>
@@ -7219,7 +7219,7 @@
     <row r="105" ht="22" customHeight="1" s="6">
       <c r="A105" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, she has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, she has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B105" s="27" t="n"/>
@@ -7235,7 +7235,7 @@
     <row r="106" ht="22" customHeight="1" s="6">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, she hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, she hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B106" s="27" t="n"/>
@@ -7395,7 +7395,7 @@
     <row r="116" ht="22" customHeight="1" s="6">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：She has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：She has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B116" s="27" t="n"/>
@@ -7411,7 +7411,7 @@
     <row r="117" ht="22" customHeight="1" s="6">
       <c r="A117" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：She hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：She hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B117" s="27" t="n"/>
@@ -7682,7 +7682,7 @@
     <row r="134" ht="22" customHeight="1" s="6">
       <c r="A134" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, you have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, you have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B134" s="27" t="n"/>
@@ -7698,7 +7698,7 @@
     <row r="135" ht="22" customHeight="1" s="6">
       <c r="A135" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, you haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, you haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B135" s="27" t="n"/>
@@ -7858,7 +7858,7 @@
     <row r="145" ht="22" customHeight="1" s="6">
       <c r="A145" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：You have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：You have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B145" s="27" t="n"/>
@@ -7874,7 +7874,7 @@
     <row r="146" ht="22" customHeight="1" s="6">
       <c r="A146" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：You haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：You haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B146" s="27" t="n"/>
@@ -8128,7 +8128,7 @@
     <row r="162" ht="22" customHeight="1" s="6">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t>正解（基本形）：No, We have never visited Kyoto.</t>
+          <t>正解（基本形）：No, we have never visited Kyoto.</t>
         </is>
       </c>
       <c r="B162" s="27" t="n"/>
@@ -8144,7 +8144,7 @@
     <row r="163" ht="22" customHeight="1" s="6">
       <c r="A163" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, We have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, we have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B163" s="27" t="n"/>
@@ -8160,7 +8160,7 @@
     <row r="164" ht="22" customHeight="1" s="6">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, We haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, we haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B164" s="27" t="n"/>
@@ -8320,7 +8320,7 @@
     <row r="174" ht="22" customHeight="1" s="6">
       <c r="A174" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：We have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：We have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B174" s="27" t="n"/>
@@ -8336,7 +8336,7 @@
     <row r="175" ht="22" customHeight="1" s="6">
       <c r="A175" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：We haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：We haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B175" s="27" t="n"/>
@@ -8606,7 +8606,7 @@
     <row r="192" ht="22" customHeight="1" s="6">
       <c r="A192" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, they have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, they have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B192" s="27" t="n"/>
@@ -8622,7 +8622,7 @@
     <row r="193" ht="22" customHeight="1" s="6">
       <c r="A193" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, they haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, they haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B193" s="27" t="n"/>
@@ -8782,7 +8782,7 @@
     <row r="203" ht="22" customHeight="1" s="6">
       <c r="A203" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：They have not visited Kyoto before.</t>
+          <t>正解（言いかえ）：They have not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B203" s="27" t="n"/>
@@ -8798,7 +8798,7 @@
     <row r="204" ht="22" customHeight="1" s="6">
       <c r="A204" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：They haven't visited Kyoto before.</t>
+          <t>正解（短縮形）：They haven't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B204" s="27" t="n"/>
@@ -9068,7 +9068,7 @@
     <row r="221" ht="22" customHeight="1" s="6">
       <c r="A221" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, he has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, he has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B221" s="27" t="n"/>
@@ -9084,7 +9084,7 @@
     <row r="222" ht="22" customHeight="1" s="6">
       <c r="A222" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, he hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, he hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B222" s="27" t="n"/>
@@ -9244,7 +9244,7 @@
     <row r="232" ht="22" customHeight="1" s="6">
       <c r="A232" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：He has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：He has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B232" s="27" t="n"/>
@@ -9260,7 +9260,7 @@
     <row r="233" ht="22" customHeight="1" s="6">
       <c r="A233" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：He hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：He hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B233" s="27" t="n"/>
@@ -9530,7 +9530,7 @@
     <row r="250" ht="22" customHeight="1" s="6">
       <c r="A250" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：No, she has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：No, she has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B250" s="27" t="n"/>
@@ -9546,7 +9546,7 @@
     <row r="251" ht="22" customHeight="1" s="6">
       <c r="A251" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, she hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：No, she hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B251" s="27" t="n"/>
@@ -9706,7 +9706,7 @@
     <row r="261" ht="22" customHeight="1" s="6">
       <c r="A261" s="11" t="inlineStr">
         <is>
-          <t>正解（言いかえ）：She has not visited Kyoto before.</t>
+          <t>正解（言いかえ）：She has not (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B261" s="27" t="n"/>
@@ -9722,7 +9722,7 @@
     <row r="262" ht="22" customHeight="1" s="6">
       <c r="A262" s="11" t="inlineStr">
         <is>
-          <t>正解（短縮形）：She hasn't visited Kyoto before.</t>
+          <t>正解（短縮形）：She hasn't (visited Kyoto before).</t>
         </is>
       </c>
       <c r="B262" s="27" t="n"/>

</xml_diff>